<commit_message>
GOODLUCK DEFENSE ft cert adjust
</commit_message>
<xml_diff>
--- a/myapp/cert_templates/Agreement_Certificate.xlsx
+++ b/myapp/cert_templates/Agreement_Certificate.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ACER\thesis_osa\myapp\cert_templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D885FDA-09C0-422B-993F-F3D7EFB3A503}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E31EC362-A30E-4030-B639-F4333C155313}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2865" yWindow="3480" windowWidth="11820" windowHeight="11295" tabRatio="500" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -72,12 +72,6 @@
     <t>TECHNOLOGICAL UNIVERSITY OF THE PHILIPPINES</t>
   </si>
   <si>
-    <t xml:space="preserve">                   CAVITE CAMPUS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">      CQT. Ave., Salawag City of Dasmariñas City, Cavite</t>
-  </si>
-  <si>
     <t>COMMUNITY SERVICE COMPLETION AGREEMENT</t>
   </si>
   <si>
@@ -91,6 +85,12 @@
   </si>
   <si>
     <t>Date Signed:</t>
+  </si>
+  <si>
+    <t>CAVITE CAMPUS</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CQT. Ave., Salawag City of Dasmariñas City, Cavite</t>
   </si>
 </sst>
 </file>
@@ -172,41 +172,41 @@
   </cellStyleXfs>
   <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -228,16 +228,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>71201</xdr:colOff>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>164422</xdr:colOff>
       <xdr:row>1</xdr:row>
-      <xdr:rowOff>32093</xdr:rowOff>
+      <xdr:rowOff>30720</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>446484</xdr:colOff>
+      <xdr:colOff>324921</xdr:colOff>
       <xdr:row>3</xdr:row>
-      <xdr:rowOff>89298</xdr:rowOff>
+      <xdr:rowOff>87925</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -256,8 +256,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="148592" y="97577"/>
-          <a:ext cx="375283" cy="378674"/>
+          <a:off x="164422" y="96662"/>
+          <a:ext cx="380307" cy="379590"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -457,34 +457,34 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A1" s="8" t="s">
+      <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="8" t="s">
+      <c r="B1" s="4" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A2" s="8" t="s">
+      <c r="A2" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="8" t="s">
+      <c r="B2" s="4" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A3" s="8" t="s">
+      <c r="A3" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="8" t="s">
+      <c r="B3" s="4" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A4" s="8" t="s">
+      <c r="A4" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="8" t="s">
+      <c r="B4" s="4" t="s">
         <v>7</v>
       </c>
     </row>
@@ -499,7 +499,7 @@
   <dimension ref="A1:E21"/>
   <sheetFormatPr defaultColWidth="0" defaultRowHeight="0" customHeight="1" zeroHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="1.140625" customWidth="1"/>
+    <col min="1" max="1" width="3.28515625" customWidth="1"/>
     <col min="2" max="2" width="27.28515625" customWidth="1"/>
     <col min="3" max="3" width="3.5703125" customWidth="1"/>
     <col min="4" max="4" width="21.28515625" customWidth="1"/>
@@ -509,101 +509,101 @@
   <sheetData>
     <row r="1" spans="2:4" ht="5.25" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="2" spans="2:4" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="B2" s="7" t="s">
+      <c r="B2" s="13" t="s">
         <v>8</v>
       </c>
-      <c r="C2" s="7"/>
-      <c r="D2" s="7"/>
+      <c r="C2" s="13"/>
+      <c r="D2" s="13"/>
     </row>
     <row r="3" spans="2:4" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="B3" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="C3" s="6"/>
-      <c r="D3" s="6"/>
+      <c r="B3" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="C3" s="10"/>
+      <c r="D3" s="10"/>
     </row>
     <row r="4" spans="2:4" ht="12" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B4" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="C4" s="5"/>
-      <c r="D4" s="5"/>
+      <c r="B4" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="C4" s="11"/>
+      <c r="D4" s="11"/>
     </row>
     <row r="5" spans="2:4" ht="12.75" x14ac:dyDescent="0.2"/>
     <row r="6" spans="2:4" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="B6" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="C6" s="4"/>
-      <c r="D6" s="4"/>
+      <c r="B6" s="12" t="s">
+        <v>9</v>
+      </c>
+      <c r="C6" s="12"/>
+      <c r="D6" s="12"/>
     </row>
     <row r="7" spans="2:4" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="B7" s="10"/>
-      <c r="C7" s="10"/>
-      <c r="D7" s="10"/>
-    </row>
-    <row r="8" spans="2:4" s="11" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B8" s="3" t="str">
+      <c r="B7" s="2"/>
+      <c r="C7" s="2"/>
+      <c r="D7" s="2"/>
+    </row>
+    <row r="8" spans="2:4" s="1" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B8" s="9" t="str">
         <f>"I " &amp; student_name &amp; " from the " &amp; program &amp; " program, understand that I must complete all pending community service hours before the end of the current semester or before applying for clearance for any academic credential. Failure to comply may result in delayed or denied clearance."</f>
         <v>I Lord Jaisson Riberal from the BET-COET program, understand that I must complete all pending community service hours before the end of the current semester or before applying for clearance for any academic credential. Failure to comply may result in delayed or denied clearance.</v>
       </c>
-      <c r="C8" s="3"/>
-      <c r="D8" s="3"/>
-    </row>
-    <row r="9" spans="2:4" s="11" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="B9" s="3"/>
-      <c r="C9" s="3"/>
-      <c r="D9" s="3"/>
-    </row>
-    <row r="10" spans="2:4" s="11" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="B10" s="3"/>
-      <c r="C10" s="3"/>
-      <c r="D10" s="3"/>
-    </row>
-    <row r="11" spans="2:4" s="11" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="B11" s="3"/>
-      <c r="C11" s="3"/>
-      <c r="D11" s="3"/>
-    </row>
-    <row r="12" spans="2:4" s="11" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="B12" s="3"/>
-      <c r="C12" s="3"/>
-      <c r="D12" s="3"/>
-    </row>
-    <row r="13" spans="2:4" s="11" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B13" s="3"/>
-      <c r="C13" s="3"/>
-      <c r="D13" s="3"/>
+      <c r="C8" s="9"/>
+      <c r="D8" s="9"/>
+    </row>
+    <row r="9" spans="2:4" s="1" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="B9" s="9"/>
+      <c r="C9" s="9"/>
+      <c r="D9" s="9"/>
+    </row>
+    <row r="10" spans="2:4" s="1" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="B10" s="9"/>
+      <c r="C10" s="9"/>
+      <c r="D10" s="9"/>
+    </row>
+    <row r="11" spans="2:4" s="1" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="B11" s="9"/>
+      <c r="C11" s="9"/>
+      <c r="D11" s="9"/>
+    </row>
+    <row r="12" spans="2:4" s="1" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="B12" s="9"/>
+      <c r="C12" s="9"/>
+      <c r="D12" s="9"/>
+    </row>
+    <row r="13" spans="2:4" s="1" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B13" s="9"/>
+      <c r="C13" s="9"/>
+      <c r="D13" s="9"/>
     </row>
     <row r="14" spans="2:4" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="B14" s="3"/>
-      <c r="C14" s="3"/>
-      <c r="D14" s="3"/>
+      <c r="B14" s="9"/>
+      <c r="C14" s="9"/>
+      <c r="D14" s="9"/>
     </row>
     <row r="15" spans="2:4" ht="12.75" x14ac:dyDescent="0.2"/>
     <row r="16" spans="2:4" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="B16" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="C16" s="2"/>
-      <c r="D16" s="12" t="str">
+      <c r="B16" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="C16" s="7"/>
+      <c r="D16" s="5" t="str">
         <f>osa_head</f>
         <v>Beverly M. de Vega</v>
       </c>
     </row>
     <row r="17" spans="2:4" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="B17" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="C17" s="1"/>
-      <c r="D17" s="9" t="s">
-        <v>14</v>
+      <c r="B17" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="C17" s="8"/>
+      <c r="D17" s="3" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="18" spans="2:4" ht="12.75" x14ac:dyDescent="0.2"/>
     <row r="19" spans="2:4" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="B19" s="13" t="s">
-        <v>15</v>
+      <c r="B19" s="6" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="20" spans="2:4" ht="12.75" x14ac:dyDescent="0.2"/>

</xml_diff>

<commit_message>
final adjust label cert
</commit_message>
<xml_diff>
--- a/myapp/cert_templates/Agreement_Certificate.xlsx
+++ b/myapp/cert_templates/Agreement_Certificate.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ACER\thesis_osa\myapp\cert_templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8A0DF3E-FCC5-4609-840D-35B0F556ACBD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78C5FD25-294E-4913-ACBE-AED0E5AA5471}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -18,7 +18,7 @@
   </sheets>
   <definedNames>
     <definedName name="osa_head">inputs!$B$4</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'Agreement Certificate'!$1:$21</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'Agreement Certificate'!$1:$23</definedName>
     <definedName name="program">inputs!$B$3</definedName>
     <definedName name="student_name">inputs!$B$2</definedName>
     <definedName name="title">inputs!$B$5</definedName>
@@ -76,15 +76,9 @@
     <t>COMMUNITY SERVICE COMPLETION AGREEMENT</t>
   </si>
   <si>
-    <t>________________________</t>
-  </si>
-  <si>
     <t>Student's Signature over Printed Name</t>
   </si>
   <si>
-    <t>Head, Office of Student Affairs</t>
-  </si>
-  <si>
     <t>Date Signed:</t>
   </si>
   <si>
@@ -95,13 +89,19 @@
   </si>
   <si>
     <t>title</t>
+  </si>
+  <si>
+    <t>Officer-In-Charge, Head, Office of Student Affairs</t>
+  </si>
+  <si>
+    <t>_______________________________</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -139,14 +139,6 @@
     </font>
     <font>
       <u/>
-      <sz val="10"/>
-      <color rgb="FF000000"/>
-      <name val="Arial"/>
-      <family val="2"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <u/>
       <sz val="9"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
@@ -174,7 +166,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -186,13 +178,7 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -209,6 +195,9 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -494,10 +483,10 @@
     </row>
     <row r="5" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="4" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
     </row>
   </sheetData>
@@ -508,7 +497,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:E23"/>
   <sheetFormatPr defaultColWidth="0" defaultRowHeight="0" customHeight="1" zeroHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="3.28515625" customWidth="1"/>
@@ -521,33 +510,33 @@
   <sheetData>
     <row r="1" spans="2:4" ht="5.25" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="2" spans="2:4" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="B2" s="10" t="s">
+      <c r="B2" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="C2" s="10"/>
-      <c r="D2" s="10"/>
+      <c r="C2" s="8"/>
+      <c r="D2" s="8"/>
     </row>
     <row r="3" spans="2:4" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="B3" s="11" t="s">
-        <v>14</v>
-      </c>
-      <c r="C3" s="11"/>
-      <c r="D3" s="11"/>
+      <c r="B3" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="C3" s="9"/>
+      <c r="D3" s="9"/>
     </row>
     <row r="4" spans="2:4" ht="12" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B4" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="C4" s="12"/>
-      <c r="D4" s="12"/>
+      <c r="B4" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="C4" s="10"/>
+      <c r="D4" s="10"/>
     </row>
     <row r="5" spans="2:4" ht="12.75" x14ac:dyDescent="0.2"/>
     <row r="6" spans="2:4" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="B6" s="13" t="s">
+      <c r="B6" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="C6" s="13"/>
-      <c r="D6" s="13"/>
+      <c r="C6" s="11"/>
+      <c r="D6" s="11"/>
     </row>
     <row r="7" spans="2:4" ht="12.75" x14ac:dyDescent="0.2">
       <c r="B7" s="2"/>
@@ -555,81 +544,96 @@
       <c r="D7" s="2"/>
     </row>
     <row r="8" spans="2:4" s="1" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B8" s="9" t="str">
+      <c r="B8" s="7" t="str">
         <f>"I " &amp; student_name &amp; " from the " &amp; program &amp; " program, understand that I must complete all pending community service hours before the end of the current semester or before applying for clearance for any academic credential. Failure to comply may result in delayed or denied clearance."</f>
         <v>I Lord Jaisson Riberal from the BET-COET program, understand that I must complete all pending community service hours before the end of the current semester or before applying for clearance for any academic credential. Failure to comply may result in delayed or denied clearance.</v>
       </c>
-      <c r="C8" s="9"/>
-      <c r="D8" s="9"/>
+      <c r="C8" s="7"/>
+      <c r="D8" s="7"/>
     </row>
     <row r="9" spans="2:4" s="1" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="B9" s="9"/>
-      <c r="C9" s="9"/>
-      <c r="D9" s="9"/>
+      <c r="B9" s="7"/>
+      <c r="C9" s="7"/>
+      <c r="D9" s="7"/>
     </row>
     <row r="10" spans="2:4" s="1" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="B10" s="9"/>
-      <c r="C10" s="9"/>
-      <c r="D10" s="9"/>
+      <c r="B10" s="7"/>
+      <c r="C10" s="7"/>
+      <c r="D10" s="7"/>
     </row>
     <row r="11" spans="2:4" s="1" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="B11" s="9"/>
-      <c r="C11" s="9"/>
-      <c r="D11" s="9"/>
+      <c r="B11" s="7"/>
+      <c r="C11" s="7"/>
+      <c r="D11" s="7"/>
     </row>
     <row r="12" spans="2:4" s="1" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="B12" s="9"/>
-      <c r="C12" s="9"/>
-      <c r="D12" s="9"/>
+      <c r="B12" s="7"/>
+      <c r="C12" s="7"/>
+      <c r="D12" s="7"/>
     </row>
     <row r="13" spans="2:4" s="1" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B13" s="9"/>
-      <c r="C13" s="9"/>
-      <c r="D13" s="9"/>
+      <c r="B13" s="7"/>
+      <c r="C13" s="7"/>
+      <c r="D13" s="7"/>
     </row>
     <row r="14" spans="2:4" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="B14" s="9"/>
-      <c r="C14" s="9"/>
-      <c r="D14" s="9"/>
+      <c r="B14" s="7"/>
+      <c r="C14" s="7"/>
+      <c r="D14" s="7"/>
     </row>
     <row r="15" spans="2:4" ht="12.75" x14ac:dyDescent="0.2"/>
     <row r="16" spans="2:4" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="B16" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="C16" s="7"/>
-      <c r="D16" s="5" t="str">
+      <c r="B16" s="12" t="str">
         <f>osa_head</f>
         <v>Beverly M. de Vega</v>
       </c>
+      <c r="C16" s="12"/>
+      <c r="D16" s="12"/>
     </row>
     <row r="17" spans="2:4" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="B17" s="8" t="s">
+      <c r="B17" s="10" t="str">
+        <f>title</f>
+        <v>Officer-In-Charge, Head, Office of Student Affairs</v>
+      </c>
+      <c r="C17" s="10"/>
+      <c r="D17" s="10"/>
+    </row>
+    <row r="18" spans="2:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="B18" s="3"/>
+      <c r="C18" s="3"/>
+      <c r="D18" s="3"/>
+    </row>
+    <row r="19" spans="2:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="B19" s="3"/>
+      <c r="C19" s="3"/>
+      <c r="D19" s="3"/>
+    </row>
+    <row r="20" spans="2:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="B20" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="C20" s="6"/>
+    </row>
+    <row r="21" spans="2:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="B21" s="6" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="22" spans="2:4" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="B22" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="C17" s="8"/>
-      <c r="D17" s="3" t="str">
-        <f>title</f>
-        <v>Head, Office of Student Affairs</v>
-      </c>
-    </row>
-    <row r="18" spans="2:4" ht="12.75" x14ac:dyDescent="0.2"/>
-    <row r="19" spans="2:4" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="B19" s="6" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="20" spans="2:4" ht="12.75" x14ac:dyDescent="0.2"/>
-    <row r="21" spans="2:4" ht="12.75" x14ac:dyDescent="0.2"/>
+    </row>
+    <row r="23" spans="2:4" ht="12.75" x14ac:dyDescent="0.2"/>
   </sheetData>
   <mergeCells count="7">
-    <mergeCell ref="B16:C16"/>
-    <mergeCell ref="B17:C17"/>
     <mergeCell ref="B8:D14"/>
     <mergeCell ref="B2:D2"/>
     <mergeCell ref="B3:D3"/>
     <mergeCell ref="B4:D4"/>
     <mergeCell ref="B6:D6"/>
+    <mergeCell ref="B17:D17"/>
+    <mergeCell ref="B16:D16"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.98402777777777795" right="0.98402777777777795" top="0.31527777777777799" bottom="0.98402777777777795" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>